<commit_message>
Match example row fonts to data cells so retyping does not inherit italic.
Remove italic example styling from the import template to avoid Excel carrying format into user-entered contact rows.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/QS_聯絡人匯入樣板.xlsx
+++ b/public/templates/QS_聯絡人匯入樣板.xlsx
@@ -42,7 +42,7 @@
     <t>• 「學術聯絡人」「雇主聯絡人」：選項欄位有下拉提示（▼），也可直接輸入；選單外文字匯入時會自動視為 Other。</t>
   </si>
   <si>
-    <t>• 灰色斜體列為範例，填寫前請刪除；可從第 2 列起填寫，最多 100 筆。</t>
+    <t>• 第 2 列為範例，填寫前請刪除；可從第 2 列起填寫，最多 100 筆。</t>
   </si>
   <si>
     <t>• 其他分頁為選項對照表（下拉選單來源），亦可手動查閱。</t>
@@ -3098,8 +3098,7 @@
   <si>
     <r>
       <rPr>
-        <i/>
-        <color rgb="FF64748B"/>
+        <color rgb="FF0F172A"/>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
       </rPr>
@@ -3107,8 +3106,7 @@
     </r>
     <r>
       <rPr>
-        <i/>
-        <color rgb="FF64748B"/>
+        <color rgb="FF0F172A"/>
         <sz val="11"/>
         <rFont val="標楷體"/>
       </rPr>
@@ -3116,8 +3114,7 @@
     </r>
     <r>
       <rPr>
-        <i/>
-        <color rgb="FF64748B"/>
+        <color rgb="FF0F172A"/>
         <sz val="11"/>
         <rFont val="Times New Roman"/>
       </rPr>
@@ -3150,7 +3147,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -3188,12 +3185,6 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-    </font>
-    <font>
-      <i/>
-      <color rgb="FF64748B"/>
       <sz val="11"/>
       <name val="Times New Roman"/>
     </font>
@@ -3238,7 +3229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3259,9 +3250,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6511,37 +6499,37 @@
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="5" t="s">
         <v>660</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="5" t="s">
         <v>661</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="5" t="s">
         <v>662</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="5" t="s">
         <v>663</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="5" t="s">
         <v>660</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="5" t="s">
         <v>601</v>
       </c>
       <c r="I2" s="7" t="s">
         <v>664</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="5" t="s">
         <v>204</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="K2" s="5" t="s">
         <v>665</v>
       </c>
     </row>
@@ -10099,34 +10087,34 @@
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="5" t="s">
         <v>660</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="5" t="s">
         <v>669</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="5" t="s">
         <v>670</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="5" t="s">
         <v>671</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="5" t="s">
         <v>601</v>
       </c>
       <c r="I2" s="7" t="s">
         <v>664</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="5" t="s">
         <v>665</v>
       </c>
     </row>

</xml_diff>